<commit_message>
style the colours page
</commit_message>
<xml_diff>
--- a/MCCC/Data/toyColours.xlsx
+++ b/MCCC/Data/toyColours.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\megan\OneDrive\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\megan\OneDrive\Documents\Crochet\MCCC\MCCC\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BC0487EA-EA95-4BCA-AC62-9CFB5B71D6D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB216CD0-1EA6-485D-99E4-B06B91721C03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0B2E8E8C-A70D-49C8-B028-F649BADB8758}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="115">
   <si>
     <t>Colour</t>
   </si>
@@ -341,9 +341,6 @@
     <t>offWhite.JPG</t>
   </si>
   <si>
-    <t>darkBrown.JPG</t>
-  </si>
-  <si>
     <t>brightRed.JPG</t>
   </si>
   <si>
@@ -384,6 +381,9 @@
   </si>
   <si>
     <t>safetyOrange.JPG</t>
+  </si>
+  <si>
+    <t>darkChocolate.JPG</t>
   </si>
 </sst>
 </file>
@@ -436,10 +436,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -759,7 +755,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B002573-DA48-4B34-B6D8-33CBAC6D2657}">
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.42578125" customWidth="1"/>
@@ -837,21 +833,21 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
+        <v>110</v>
+      </c>
+      <c r="C7" t="s">
         <v>111</v>
-      </c>
-      <c r="C7" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
+        <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -859,10 +855,10 @@
         <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="C9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -870,10 +866,10 @@
         <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="C10" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -881,21 +877,21 @@
         <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="C11" t="s">
-        <v>62</v>
+        <v>92</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B12" t="s">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="C12" t="s">
-        <v>92</v>
+        <v>63</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -903,10 +899,10 @@
         <v>9</v>
       </c>
       <c r="B13" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="C13" t="s">
-        <v>63</v>
+        <v>93</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -914,10 +910,10 @@
         <v>9</v>
       </c>
       <c r="B14" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="C14" t="s">
-        <v>93</v>
+        <v>64</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -925,10 +921,10 @@
         <v>9</v>
       </c>
       <c r="B15" t="s">
-        <v>10</v>
+        <v>49</v>
       </c>
       <c r="C15" t="s">
-        <v>64</v>
+        <v>94</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -936,10 +932,10 @@
         <v>9</v>
       </c>
       <c r="B16" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C16" t="s">
-        <v>94</v>
+        <v>65</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -947,21 +943,21 @@
         <v>9</v>
       </c>
       <c r="B17" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="C17" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B18" t="s">
-        <v>53</v>
+        <v>31</v>
       </c>
       <c r="C18" t="s">
-        <v>66</v>
+        <v>95</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -969,10 +965,10 @@
         <v>11</v>
       </c>
       <c r="B19" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="C19" t="s">
-        <v>95</v>
+        <v>67</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -980,21 +976,21 @@
         <v>11</v>
       </c>
       <c r="B20" t="s">
-        <v>11</v>
+        <v>112</v>
       </c>
       <c r="C20" t="s">
-        <v>67</v>
+        <v>113</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B21" t="s">
-        <v>113</v>
+        <v>35</v>
       </c>
       <c r="C21" t="s">
-        <v>114</v>
+        <v>68</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -1002,10 +998,10 @@
         <v>12</v>
       </c>
       <c r="B22" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="C22" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -1013,10 +1009,10 @@
         <v>12</v>
       </c>
       <c r="B23" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="C23" t="s">
-        <v>69</v>
+        <v>96</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -1024,10 +1020,10 @@
         <v>12</v>
       </c>
       <c r="B24" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="C24" t="s">
-        <v>96</v>
+        <v>70</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -1035,10 +1031,10 @@
         <v>12</v>
       </c>
       <c r="B25" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="C25" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -1046,10 +1042,10 @@
         <v>12</v>
       </c>
       <c r="B26" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="C26" t="s">
-        <v>71</v>
+        <v>97</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -1057,21 +1053,21 @@
         <v>12</v>
       </c>
       <c r="B27" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C27" t="s">
-        <v>97</v>
+        <v>72</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B28" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C28" t="s">
-        <v>72</v>
+        <v>98</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -1079,10 +1075,10 @@
         <v>14</v>
       </c>
       <c r="B29" t="s">
-        <v>50</v>
+        <v>14</v>
       </c>
       <c r="C29" t="s">
-        <v>98</v>
+        <v>73</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -1090,10 +1086,10 @@
         <v>14</v>
       </c>
       <c r="B30" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="C30" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -1101,10 +1097,10 @@
         <v>14</v>
       </c>
       <c r="B31" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C31" t="s">
-        <v>74</v>
+        <v>98</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -1112,10 +1108,10 @@
         <v>14</v>
       </c>
       <c r="B32" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C32" t="s">
-        <v>98</v>
+        <v>76</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -1123,10 +1119,10 @@
         <v>14</v>
       </c>
       <c r="B33" t="s">
-        <v>44</v>
+        <v>15</v>
       </c>
       <c r="C33" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -1134,10 +1130,10 @@
         <v>14</v>
       </c>
       <c r="B34" t="s">
-        <v>15</v>
+        <v>106</v>
       </c>
       <c r="C34" t="s">
-        <v>77</v>
+        <v>107</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -1145,21 +1141,21 @@
         <v>14</v>
       </c>
       <c r="B35" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C35" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B36" t="s">
-        <v>109</v>
+        <v>16</v>
       </c>
       <c r="C36" t="s">
-        <v>110</v>
+        <v>78</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -1167,10 +1163,10 @@
         <v>16</v>
       </c>
       <c r="B37" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C37" t="s">
-        <v>78</v>
+        <v>99</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -1178,21 +1174,21 @@
         <v>16</v>
       </c>
       <c r="B38" t="s">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="C38" t="s">
-        <v>99</v>
+        <v>79</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B39" t="s">
-        <v>51</v>
+        <v>30</v>
       </c>
       <c r="C39" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -1200,10 +1196,10 @@
         <v>18</v>
       </c>
       <c r="B40" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="C40" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
@@ -1211,21 +1207,21 @@
         <v>18</v>
       </c>
       <c r="B41" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="C41" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="B42" t="s">
-        <v>43</v>
+        <v>24</v>
       </c>
       <c r="C42" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
@@ -1233,10 +1229,10 @@
         <v>23</v>
       </c>
       <c r="B43" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C43" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -1244,10 +1240,10 @@
         <v>23</v>
       </c>
       <c r="B44" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="C44" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -1255,10 +1251,10 @@
         <v>23</v>
       </c>
       <c r="B45" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C45" t="s">
-        <v>85</v>
+        <v>114</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
@@ -1266,10 +1262,10 @@
         <v>23</v>
       </c>
       <c r="B46" t="s">
-        <v>39</v>
+        <v>102</v>
       </c>
       <c r="C46" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
@@ -1285,13 +1281,13 @@
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B48" t="s">
-        <v>104</v>
+        <v>29</v>
       </c>
       <c r="C48" t="s">
-        <v>106</v>
+        <v>86</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -1299,10 +1295,10 @@
         <v>28</v>
       </c>
       <c r="B49" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="C49" t="s">
-        <v>86</v>
+        <v>100</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -1310,10 +1306,10 @@
         <v>28</v>
       </c>
       <c r="B50" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C50" t="s">
-        <v>101</v>
+        <v>87</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -1321,21 +1317,21 @@
         <v>28</v>
       </c>
       <c r="B51" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C51" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="B52" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="C52" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
@@ -1343,10 +1339,10 @@
         <v>38</v>
       </c>
       <c r="B53" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="C53" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
@@ -1354,31 +1350,20 @@
         <v>38</v>
       </c>
       <c r="B54" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="C54" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="B55" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C55" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>55</v>
-      </c>
-      <c r="B56" t="s">
-        <v>55</v>
-      </c>
-      <c r="C56" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>